<commit_message>
feat: adiciona pipeline de CI/CD, Circuit Breaker, logs críticos e gravação na planilha mestra
</commit_message>
<xml_diff>
--- a/02_AUTOMACAO_ECOS/data/controle_mestre_ecos.xlsx
+++ b/02_AUTOMACAO_ECOS/data/controle_mestre_ecos.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controle_Mestre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,21 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,100 +413,318 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="25" customWidth="1" min="15" max="15"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Codigo_ECO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Titulo_Alteracao</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Area_Solicitante</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Nome_Engenheiro_Responsavel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Email_Solicitante</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Data_Recebimento</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Nivel_Prioridade</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status_Atual</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Justificativa_Tecnica</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Codigo_Item_Afetado</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Categoria_Mudanca</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Impacto_Custos</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Estimativa_Orcamento</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Unidade_Fabril</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Data_Implementacao_Alvo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Status_Automacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ECO-00126</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Alteração dimensional do suporte</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Engenharia</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>carlos.lima@matriz.example</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>SUP-778</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>3500</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>PENDENTE_VALIDACAO_HUMANA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ECO-00127</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Atualização urgente de firmware</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Engenharia de Software</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bruno Costa</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bruno.costa@matriz.example</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Correção emergencial de firmware.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>FW-900</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>-500</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>BLOQUEADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ECO-00125</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Atualização do layout do módulo de refrigeração</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Engenharia</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ana.souza@matriz.example</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Adequação do posicionamento do componente para melhoria de montagem.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ITEM-REF-220</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige ambiente local e valida execução da automação ECO
</commit_message>
<xml_diff>
--- a/02_AUTOMACAO_ECOS/data/controle_mestre_ecos.xlsx
+++ b/02_AUTOMACAO_ECOS/data/controle_mestre_ecos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -707,8 +707,10 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="M4" t="n">
-        <v>0</v>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -721,236 +723,6 @@
         </is>
       </c>
       <c r="P4" t="inlineStr">
-        <is>
-          <t>REGISTRADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ECO-00126</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Alteração dimensional do suporte</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Engenharia</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Carlos Lima</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>carlos.lima@matriz.example</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Média</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>SUP-778</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Componente</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>3500</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Manaus</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>PENDENTE_VALIDACAO_HUMANA</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ECO-00127</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Atualização urgente de firmware</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Engenharia de Software</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Bruno Costa</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>bruno.costa@matriz.example</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Correção emergencial de firmware.</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>FW-900</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Software</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>-500</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Manaus</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>BLOQUEADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ECO-00125</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Atualização do layout do módulo de refrigeração</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Engenharia</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Ana Souza</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ana.souza@matriz.example</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Adequação do posicionamento do componente para melhoria de montagem.</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>ITEM-REF-220</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Layout</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Manaus</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
         <is>
           <t>REGISTRADO</t>
         </is>

</xml_diff>

<commit_message>
feat: adiciona criacao automatica de pastas para portabilidade
</commit_message>
<xml_diff>
--- a/02_AUTOMACAO_ECOS/data/controle_mestre_ecos.xlsx
+++ b/02_AUTOMACAO_ECOS/data/controle_mestre_ecos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -707,22 +707,478 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ECO-00126</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Alteração dimensional do suporte</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Engenharia</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>carlos.lima@matriz.example</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SUP-778</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>ERRO_SISTEMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ECO-00127</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Atualização urgente de firmware</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Engenharia de Software</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Bruno Costa</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>bruno.costa@matriz.example</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Correção emergencial de firmware.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>FW-900</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>-500</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>BLOQUEADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ECO-00125</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Atualização do layout do módulo de refrigeração</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Engenharia</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ana.souza@matriz.example</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Adequação do posicionamento do componente para melhoria de montagem.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>ITEM-REF-220</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>ERRO_SISTEMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ECO-00126</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Alteração dimensional do suporte</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Engenharia</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>carlos.lima@matriz.example</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SUP-778</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>3500</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>PENDENTE_VALIDACAO_HUMANA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ECO-00127</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Atualização urgente de firmware</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Engenharia de Software</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Bruno Costa</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>bruno.costa@matriz.example</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Correção emergencial de firmware.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>FW-900</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>-500</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>BLOQUEADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ECO-00125</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Atualização do layout do módulo de refrigeração</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Engenharia</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ana Souza</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ana.souza@matriz.example</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Adequação do posicionamento do componente para melhoria de montagem.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ITEM-REF-220</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Manaus</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>REGISTRADO</t>
         </is>

</xml_diff>